<commit_message>
Normalize experimental data and rebuild workbook
</commit_message>
<xml_diff>
--- a/sources/Datos_Ema_Serrana_INN.xlsx
+++ b/sources/Datos_Ema_Serrana_INN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/agustinsellanes/Repos/festuca_probabilistic_analysis/sources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD29BC1-E101-EF4A-AF55-E86DAE7A8559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20B5EA05-00A0-1345-A614-ED4F4DA7CFAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1256,10 +1256,10 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1617,11 +1617,11 @@
       <c r="A5" s="58"/>
       <c r="B5" s="58"/>
       <c r="C5" s="95"/>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="94"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="91"/>
+      <c r="F5" s="91"/>
+      <c r="G5" s="91"/>
+      <c r="H5" s="92"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="60" t="s">
@@ -1650,62 +1650,62 @@
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="58"/>
       <c r="B7" s="58"/>
-      <c r="C7" s="91"/>
-      <c r="D7" s="91"/>
-      <c r="E7" s="91"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="91"/>
-      <c r="H7" s="91"/>
+      <c r="C7" s="93"/>
+      <c r="D7" s="93"/>
+      <c r="E7" s="93"/>
+      <c r="F7" s="93"/>
+      <c r="G7" s="93"/>
+      <c r="H7" s="93"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="58"/>
       <c r="B8" s="58"/>
-      <c r="C8" s="91"/>
-      <c r="D8" s="91"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="91"/>
-      <c r="G8" s="91"/>
-      <c r="H8" s="91"/>
+      <c r="C8" s="93"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="58"/>
       <c r="B9" s="58"/>
-      <c r="C9" s="91"/>
-      <c r="D9" s="91"/>
-      <c r="E9" s="91"/>
-      <c r="F9" s="91"/>
-      <c r="G9" s="91"/>
-      <c r="H9" s="91"/>
+      <c r="C9" s="93"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="93"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="58"/>
       <c r="B10" s="58"/>
-      <c r="C10" s="91"/>
-      <c r="D10" s="91"/>
-      <c r="E10" s="91"/>
-      <c r="F10" s="91"/>
-      <c r="G10" s="91"/>
-      <c r="H10" s="91"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
+      <c r="H10" s="93"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="58"/>
       <c r="B11" s="58"/>
-      <c r="C11" s="92"/>
-      <c r="D11" s="92"/>
-      <c r="E11" s="92"/>
-      <c r="F11" s="92"/>
-      <c r="G11" s="92"/>
-      <c r="H11" s="92"/>
+      <c r="C11" s="94"/>
+      <c r="D11" s="94"/>
+      <c r="E11" s="94"/>
+      <c r="F11" s="94"/>
+      <c r="G11" s="94"/>
+      <c r="H11" s="94"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="61"/>
       <c r="B12" s="58"/>
       <c r="C12" s="90"/>
-      <c r="D12" s="93"/>
-      <c r="E12" s="93"/>
-      <c r="F12" s="93"/>
-      <c r="G12" s="93"/>
-      <c r="H12" s="94"/>
+      <c r="D12" s="91"/>
+      <c r="E12" s="91"/>
+      <c r="F12" s="91"/>
+      <c r="G12" s="91"/>
+      <c r="H12" s="92"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="58"/>
@@ -1732,62 +1732,62 @@
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="58"/>
       <c r="B14" s="58"/>
-      <c r="C14" s="91"/>
-      <c r="D14" s="91"/>
-      <c r="E14" s="91"/>
-      <c r="F14" s="91"/>
-      <c r="G14" s="91"/>
-      <c r="H14" s="91"/>
+      <c r="C14" s="93"/>
+      <c r="D14" s="93"/>
+      <c r="E14" s="93"/>
+      <c r="F14" s="93"/>
+      <c r="G14" s="93"/>
+      <c r="H14" s="93"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="58"/>
       <c r="B15" s="58"/>
-      <c r="C15" s="91"/>
-      <c r="D15" s="91"/>
-      <c r="E15" s="91"/>
-      <c r="F15" s="91"/>
-      <c r="G15" s="91"/>
-      <c r="H15" s="91"/>
+      <c r="C15" s="93"/>
+      <c r="D15" s="93"/>
+      <c r="E15" s="93"/>
+      <c r="F15" s="93"/>
+      <c r="G15" s="93"/>
+      <c r="H15" s="93"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="58"/>
       <c r="B16" s="58"/>
-      <c r="C16" s="91"/>
-      <c r="D16" s="91"/>
-      <c r="E16" s="91"/>
-      <c r="F16" s="91"/>
-      <c r="G16" s="91"/>
-      <c r="H16" s="91"/>
+      <c r="C16" s="93"/>
+      <c r="D16" s="93"/>
+      <c r="E16" s="93"/>
+      <c r="F16" s="93"/>
+      <c r="G16" s="93"/>
+      <c r="H16" s="93"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="58"/>
       <c r="B17" s="58"/>
-      <c r="C17" s="91"/>
-      <c r="D17" s="91"/>
-      <c r="E17" s="91"/>
-      <c r="F17" s="91"/>
-      <c r="G17" s="91"/>
-      <c r="H17" s="91"/>
+      <c r="C17" s="93"/>
+      <c r="D17" s="93"/>
+      <c r="E17" s="93"/>
+      <c r="F17" s="93"/>
+      <c r="G17" s="93"/>
+      <c r="H17" s="93"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="58"/>
       <c r="B18" s="58"/>
-      <c r="C18" s="92"/>
-      <c r="D18" s="92"/>
-      <c r="E18" s="92"/>
-      <c r="F18" s="92"/>
-      <c r="G18" s="92"/>
-      <c r="H18" s="92"/>
+      <c r="C18" s="94"/>
+      <c r="D18" s="94"/>
+      <c r="E18" s="94"/>
+      <c r="F18" s="94"/>
+      <c r="G18" s="94"/>
+      <c r="H18" s="94"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="58"/>
       <c r="B19" s="58"/>
       <c r="C19" s="90"/>
-      <c r="D19" s="93"/>
-      <c r="E19" s="93"/>
-      <c r="F19" s="93"/>
-      <c r="G19" s="93"/>
-      <c r="H19" s="94"/>
+      <c r="D19" s="91"/>
+      <c r="E19" s="91"/>
+      <c r="F19" s="91"/>
+      <c r="G19" s="91"/>
+      <c r="H19" s="92"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="58"/>
@@ -1814,62 +1814,62 @@
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="58"/>
       <c r="B21" s="58"/>
-      <c r="C21" s="91"/>
-      <c r="D21" s="91"/>
-      <c r="E21" s="91"/>
-      <c r="F21" s="91"/>
-      <c r="G21" s="91"/>
-      <c r="H21" s="91"/>
+      <c r="C21" s="93"/>
+      <c r="D21" s="93"/>
+      <c r="E21" s="93"/>
+      <c r="F21" s="93"/>
+      <c r="G21" s="93"/>
+      <c r="H21" s="93"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="58"/>
       <c r="B22" s="58"/>
-      <c r="C22" s="91"/>
-      <c r="D22" s="91"/>
-      <c r="E22" s="91"/>
-      <c r="F22" s="91"/>
-      <c r="G22" s="91"/>
-      <c r="H22" s="91"/>
+      <c r="C22" s="93"/>
+      <c r="D22" s="93"/>
+      <c r="E22" s="93"/>
+      <c r="F22" s="93"/>
+      <c r="G22" s="93"/>
+      <c r="H22" s="93"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="58"/>
       <c r="B23" s="58"/>
-      <c r="C23" s="91"/>
-      <c r="D23" s="91"/>
-      <c r="E23" s="91"/>
-      <c r="F23" s="91"/>
-      <c r="G23" s="91"/>
-      <c r="H23" s="91"/>
+      <c r="C23" s="93"/>
+      <c r="D23" s="93"/>
+      <c r="E23" s="93"/>
+      <c r="F23" s="93"/>
+      <c r="G23" s="93"/>
+      <c r="H23" s="93"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="58"/>
       <c r="B24" s="58"/>
-      <c r="C24" s="91"/>
-      <c r="D24" s="91"/>
-      <c r="E24" s="91"/>
-      <c r="F24" s="91"/>
-      <c r="G24" s="91"/>
-      <c r="H24" s="91"/>
+      <c r="C24" s="93"/>
+      <c r="D24" s="93"/>
+      <c r="E24" s="93"/>
+      <c r="F24" s="93"/>
+      <c r="G24" s="93"/>
+      <c r="H24" s="93"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="58"/>
       <c r="B25" s="58"/>
-      <c r="C25" s="92"/>
-      <c r="D25" s="92"/>
-      <c r="E25" s="92"/>
-      <c r="F25" s="92"/>
-      <c r="G25" s="92"/>
-      <c r="H25" s="92"/>
+      <c r="C25" s="94"/>
+      <c r="D25" s="94"/>
+      <c r="E25" s="94"/>
+      <c r="F25" s="94"/>
+      <c r="G25" s="94"/>
+      <c r="H25" s="94"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="58"/>
       <c r="B26" s="58"/>
       <c r="C26" s="90"/>
-      <c r="D26" s="93"/>
-      <c r="E26" s="93"/>
-      <c r="F26" s="93"/>
-      <c r="G26" s="93"/>
-      <c r="H26" s="94"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="91"/>
+      <c r="F26" s="91"/>
+      <c r="G26" s="91"/>
+      <c r="H26" s="92"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="58"/>
@@ -1896,65 +1896,78 @@
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="58"/>
       <c r="B28" s="58"/>
-      <c r="C28" s="91"/>
-      <c r="D28" s="91"/>
-      <c r="E28" s="91"/>
-      <c r="F28" s="91"/>
-      <c r="G28" s="91"/>
-      <c r="H28" s="91"/>
+      <c r="C28" s="93"/>
+      <c r="D28" s="93"/>
+      <c r="E28" s="93"/>
+      <c r="F28" s="93"/>
+      <c r="G28" s="93"/>
+      <c r="H28" s="93"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="58"/>
       <c r="B29" s="58"/>
-      <c r="C29" s="91"/>
-      <c r="D29" s="91"/>
-      <c r="E29" s="91"/>
-      <c r="F29" s="91"/>
-      <c r="G29" s="91"/>
-      <c r="H29" s="91"/>
+      <c r="C29" s="93"/>
+      <c r="D29" s="93"/>
+      <c r="E29" s="93"/>
+      <c r="F29" s="93"/>
+      <c r="G29" s="93"/>
+      <c r="H29" s="93"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="58"/>
       <c r="B30" s="58"/>
-      <c r="C30" s="91"/>
-      <c r="D30" s="91"/>
-      <c r="E30" s="91"/>
-      <c r="F30" s="91"/>
-      <c r="G30" s="91"/>
-      <c r="H30" s="91"/>
+      <c r="C30" s="93"/>
+      <c r="D30" s="93"/>
+      <c r="E30" s="93"/>
+      <c r="F30" s="93"/>
+      <c r="G30" s="93"/>
+      <c r="H30" s="93"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="58"/>
       <c r="B31" s="58"/>
-      <c r="C31" s="91"/>
-      <c r="D31" s="91"/>
-      <c r="E31" s="91"/>
-      <c r="F31" s="91"/>
-      <c r="G31" s="91"/>
-      <c r="H31" s="91"/>
+      <c r="C31" s="93"/>
+      <c r="D31" s="93"/>
+      <c r="E31" s="93"/>
+      <c r="F31" s="93"/>
+      <c r="G31" s="93"/>
+      <c r="H31" s="93"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="58"/>
       <c r="B32" s="58"/>
-      <c r="C32" s="92"/>
-      <c r="D32" s="92"/>
-      <c r="E32" s="92"/>
-      <c r="F32" s="92"/>
-      <c r="G32" s="92"/>
-      <c r="H32" s="92"/>
+      <c r="C32" s="94"/>
+      <c r="D32" s="94"/>
+      <c r="E32" s="94"/>
+      <c r="F32" s="94"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="94"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="58"/>
       <c r="B33" s="58"/>
       <c r="C33" s="90"/>
-      <c r="D33" s="93"/>
-      <c r="E33" s="93"/>
-      <c r="F33" s="93"/>
-      <c r="G33" s="93"/>
-      <c r="H33" s="94"/>
+      <c r="D33" s="91"/>
+      <c r="E33" s="91"/>
+      <c r="F33" s="91"/>
+      <c r="G33" s="91"/>
+      <c r="H33" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="C6:C11"/>
+    <mergeCell ref="D6:D11"/>
+    <mergeCell ref="F6:F11"/>
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="E6:E11"/>
+    <mergeCell ref="G6:G11"/>
+    <mergeCell ref="D13:D18"/>
+    <mergeCell ref="C27:C32"/>
+    <mergeCell ref="F13:F18"/>
+    <mergeCell ref="E27:E32"/>
+    <mergeCell ref="H13:H18"/>
+    <mergeCell ref="H20:H25"/>
     <mergeCell ref="C33:H33"/>
     <mergeCell ref="F27:F32"/>
     <mergeCell ref="H27:H32"/>
@@ -1971,19 +1984,6 @@
     <mergeCell ref="G13:G18"/>
     <mergeCell ref="F20:F25"/>
     <mergeCell ref="C19:H19"/>
-    <mergeCell ref="D13:D18"/>
-    <mergeCell ref="C27:C32"/>
-    <mergeCell ref="F13:F18"/>
-    <mergeCell ref="E27:E32"/>
-    <mergeCell ref="H13:H18"/>
-    <mergeCell ref="H20:H25"/>
-    <mergeCell ref="C6:C11"/>
-    <mergeCell ref="D6:D11"/>
-    <mergeCell ref="F6:F11"/>
-    <mergeCell ref="C12:H12"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="E6:E11"/>
-    <mergeCell ref="G6:G11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2045,7 +2045,7 @@
         <v>45820</v>
       </c>
       <c r="H3" s="64">
-        <v>45869</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -2065,7 +2065,7 @@
         <v>45835</v>
       </c>
       <c r="H4" s="64">
-        <v>45869</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -2322,7 +2322,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="64">
-        <v>46238</v>
+        <v>45873</v>
       </c>
       <c r="B22" s="58" t="s">
         <v>40</v>
@@ -2350,7 +2350,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="64">
-        <v>46281</v>
+        <v>45916</v>
       </c>
       <c r="B24" s="58" t="s">
         <v>42</v>
@@ -2392,7 +2392,7 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="66">
-        <v>46338</v>
+        <v>45973</v>
       </c>
       <c r="B27" s="58" t="s">
         <v>175</v>
@@ -8773,8 +8773,8 @@
       <c r="I5" s="100" t="s">
         <v>111</v>
       </c>
-      <c r="J5" s="93"/>
-      <c r="K5" s="94"/>
+      <c r="J5" s="91"/>
+      <c r="K5" s="92"/>
       <c r="L5" s="48" t="s">
         <v>112</v>
       </c>

</xml_diff>